<commit_message>
Soru metinlerine gebelik şekeri bağlamını ekle ve CAS'ı soru başına madde haritasıyla puanla.
Puanlanmayan CAS maddesi NULL (eksik veri) kaydedilir; karşılaştırma cas_pct ile yapılır.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/GDM_Final_30_Soru_Birlesik.xlsx
+++ b/data/GDM_Final_30_Soru_Birlesik.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final 30 Soru Havuzu" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Özet İstatistikler" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Sorgu Planı" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Final 30 Soru Havuzu" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Özet İstatistikler" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="API Sorgu Planı" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -256,6 +256,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -621,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -629,6 +635,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -664,6 +671,11 @@
           <t>SORU METNİ</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>BAĞLAM EKLENMEDEN ÖNCEKİ METİN</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="65" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -715,6 +727,11 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Karbonhidratı nasıl ve ne kadar tüketebilirim, hangileri daha güvenli?</t>
+        </is>
+      </c>
+      <c r="F4" s="38" t="inlineStr">
+        <is>
           <t>Karbonhidratı nasıl ve ne kadar tüketebilirim, hangileri daha güvenli?</t>
         </is>
       </c>
@@ -742,6 +759,11 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Canım tatlı çektiğinde ne yapabilirim? Her akşam dondurma yesem, arkasından yürüyüş yapsam yiyebilir miyim? Bir kare çikolata veya küçük bir kase puding sıkıntı oluşturur mu?</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
           <t>Canım tatlı çektiğinde ne yapabilirim? Her akşam dondurma yesem, arkasından yürüyüş yapsam yiyebilir miyim? Bir kare çikolata veya küçük bir kase puding sıkıntı oluşturur mu?</t>
         </is>
       </c>
@@ -769,6 +791,11 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Hangi meyveleri yiyebilirim, hangilerinin şekeri daha yüksek? Örneğin karpuzdan günde kaç dilim yiyebilirim?</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
           <t>Hangi meyveleri yiyebilirim, hangilerinin şekeri daha yüksek? Örneğin karpuzdan günde kaç dilim yiyebilirim?</t>
         </is>
       </c>
@@ -796,6 +823,11 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Meyveli soda içebilir miyim? Kramplarım için sade soda içemiyorum, meyveli olanı da şekerimi yükseltir mi?</t>
+        </is>
+      </c>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
           <t>Meyveli soda içebilir miyim? Şeker hastasıyken kramplarım için sade soda içemiyorum, meyveli olanı da şekerimi yükseltir mi?</t>
         </is>
       </c>
@@ -823,6 +855,11 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Oruçken sahurda ve iftarda yediklerim bebeğim için yeterli besini sağlar mı? İftardan sahura kadar çok yiyecek tüketemiyorum, uzun süre tok tutması için ne yiyebilirim?</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
           <t>Oruçken sahurda ve iftarda yediklerim bebeğim için yeterli besini sağlar mı? İftardan sahura kadar çok yiyecek tüketemiyorum, uzun süre tok tutması için ne yiyebilirim?</t>
         </is>
       </c>
@@ -850,6 +887,11 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Oruç sırasında uzun süre aç kalmam kan şekeri dengemi bozar mı, bebeğime zarar verir mi? Herhangi bir şikayetim olmasa bile bebeğe zararı olur mu?</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
           <t>Oruç sırasında uzun süre aç kalmam kan şekeri dengemi bozar mı, bebeğime zarar verir mi? Herhangi bir şikayetim olmasa bile bebeğe zararı olur mu?</t>
         </is>
       </c>
@@ -877,6 +919,11 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Ramazan ayında 2 gün oruç tutabildim, baş dönmesi ve titreme oldu tutamadım, tutsam sorun olur muydu? Oruç tutarken aç kalırsam bayılır mıyım?</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
           <t>Ramazan ayında 2 gün oruç tutabildim, baş dönmesi ve titreme oldu tutamadım, tutsam sorun olur muydu? Oruç tutarken aç kalırsam bayılır mıyım?</t>
         </is>
       </c>
@@ -931,6 +978,11 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
+          <t>Hamileliğimde gebelik şekeri çıkmıştı, yeni doğum yaptım. Lohusa döneminde şekere ne kadar dikkat etmeliyim, şeker takipleri ne kadar sürer, diyet devam eder mi? İstediğim tatlı ve yemekleri tüketebilir miyim?</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
           <t>Lohusa döneminde şekere ne kadar dikkat etmeliyim, şeker takipleri ne kadar sürer, diyet devam eder mi? İstediğim tatlı ve yemekleri tüketebilir miyim?</t>
         </is>
       </c>
@@ -958,6 +1010,11 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
+          <t>Hamileliğimde gebelik şekeri çıkmıştı. Yeni doğum yaptım, kaynanam sütüm artsın diye sürekli lohusa şerbeti içmem gerektiğini söylüyor ama ben zararlı olacağını düşünüyorum, içmeli miyim? Doğum sonrası yapılan lapa şekerimi yükseltir mi?</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
           <t>Yeni doğum yaptım, kaynanam sütüm artsın diye sürekli lohusa şerbeti içmem gerektiğini söylüyor ama ben zararlı olacağını düşünüyorum, içmeli miyim? Doğum sonrası yapılan lapa şekerimi yükseltir mi?</t>
         </is>
       </c>
@@ -985,6 +1042,11 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
+          <t>Hamileliğimde gebelik şekeri çıkmıştı, şimdi bebeğimi emziriyorum. Emzirme döneminde şekerli besinler sütü arttırır mı?</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
           <t>Emzirme döneminde şekerli besinler sütü arttırır mı?</t>
         </is>
       </c>
@@ -1012,6 +1074,11 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
+          <t>Hamileliğimde gebelik şekeri çıkmıştı. Doğum yaptıktan sonra artık şeker hastası mı olacağım, yoksa doğumla geçecek mi? Şeker düzelsin diye sürekli spor yapıp hızla kilo mu vermem gerekir?</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
           <t>Doğum yaptıktan sonra artık şeker hastası mı olacağım, yoksa doğumla geçecek mi? Şeker düzelsin diye sürekli spor yapıp hızla kilo mu vermem gerekir?</t>
         </is>
       </c>
@@ -1039,6 +1106,11 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
+          <t>Hamileliğimde gebelik şekeri çıktığı için bebeğim de şeker hastası olacak mı, çocukta kalıcı olur mu?</t>
+        </is>
+      </c>
+      <c r="F16" s="38" t="inlineStr">
+        <is>
           <t>Ben şeker hastası olduğum için bebeğim de şeker hastası olacak mı, çocukta kalıcı olur mu?</t>
         </is>
       </c>
@@ -1066,6 +1138,11 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
+          <t>Gebelik şekeri tanısı aldım, şeker ölçüm cihazı yazıldı, SGK karşılıyor mu yoksa ben ne kadar ücretle satın alabilirim? Cihazım bozulursa sigortam karşılayacak mı?</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
           <t>Şeker tanısı aldım, şeker ölçüm cihazı yazıldı, SGK karşılıyor mu yoksa ben ne kadar ücretle satın alabilirim? Cihazım bozulursa sigortam karşılayacak mı?</t>
         </is>
       </c>
@@ -1093,6 +1170,11 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Şeker ölçümü için kullandığım stikler yetmedi, yazdırdım ama eczane süresi dolmadığı için para ile almam gerektiğini söyledi, ben de stikler yetsin diye sabahları açlık şekerimi ölçmeyi bıraktım, bu doğru mu? Sigortam yok, insülinleri de paralı mı alacağım?</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
           <t>Şeker ölçümü için kullandığım stikler yetmedi, yazdırdım ama eczane süresi dolmadığı için para ile almam gerektiğini söyledi, ben de stikler yetsin diye sabahları açlık şekerimi ölçmeyi bıraktım, bu doğru mu? Sigortam yok, insülinleri de paralı mı alacağım?</t>
         </is>
       </c>
@@ -1120,6 +1202,11 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Aile ve sosyal ortamda diyetime uymakta zorlanıyorum, nasıl denge kurabilirim?</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
           <t>Aile ve sosyal ortamda diyetime uymakta zorlanıyorum, nasıl denge kurabilirim?</t>
         </is>
       </c>
@@ -1147,6 +1234,11 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Misafirlikte ısrar ediliyor, canım çeker gibi ne yiyebilirim ne kadar ölçekte? Bayramda tatlıyı fazla kaçırırsam nasıl telafi edebilirim, bebeğim zarar görmüş müdür?</t>
+        </is>
+      </c>
+      <c r="F20" s="38" t="inlineStr">
+        <is>
           <t>Misafirlikte ısrar ediliyor, canım çeker gibi ne yiyebilirim ne kadar ölçekte? Bayramda tatlıyı fazla kaçırırsam nasıl telafi edebilirim, bebeğim zarar görmüş müdür?</t>
         </is>
       </c>
@@ -1174,6 +1266,11 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Aşerdiğim yiyeceğin diyetimi bozduğunu bildiğim halde yiyebilir miyim? Yememem gereken bir besinin muadilini yemek yeterli gelmiyor, bir parça yesem çok sorun olur mu?</t>
+        </is>
+      </c>
+      <c r="F21" s="38" t="inlineStr">
+        <is>
           <t>Aşerdiğim yiyeceğin diyetimi bozduğunu bildiğim halde yiyebilir miyim? Yememem gereken bir besinin muadilini yemek yeterli gelmiyor, bir parça yesem çok sorun olur mu?</t>
         </is>
       </c>
@@ -1201,6 +1298,11 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
+          <t>Gebelik şekerim olduğu için diyet yapıyorum, ailem sürekli bana bir şeyler yedirmeye çalışıyor, 'sen gebesin bebek aç kalır' diyor. Eşimin akrabaları da psikolojik baskı yapıyor. Kaynanam 'tatlı yemek istediğinde limon ye geçer' diyor, bu doğru mu?</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
           <t>Diyet yaptığım için ailem sürekli bana bir şeyler yedirmeye çalışıyor, 'sen gebesin bebek aç kalır' diyor. Eşimin akrabaları da psikolojik baskı yapıyor. Kaynanam 'tatlı yemek istediğinde limon ye geçer' diyor, bu doğru mu?</t>
         </is>
       </c>
@@ -1228,6 +1330,11 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Komşularla gün yaparken çayın yanında tatlı yiyemiyorum. En azından markette satılan tatlandırıcılardan koysam olur mu? Hamilelikte tatlandırıcı kullanmak bebeğe zarar verir mi?</t>
+        </is>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
           <t>Komşularla gün yaparken çayın yanında tatlı yiyemiyorum. En azından markette satılan tatlandırıcılardan koysam olur mu? Hamilelikte tatlandırıcı kullanmak bebeğe zarar verir mi?</t>
         </is>
       </c>
@@ -1255,6 +1362,11 @@
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Kayınvalidem sürekli yemeklerden sonra meyve yemem gerektiğini, bebeğe faydası olacağını söyleyip duruyor. Bu şekerimi yükseltir mi, bebeğime zararı olur mu?</t>
+        </is>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
           <t>Kayınvalidem sürekli yemeklerden sonra meyve yemem gerektiğini, bebeğe faydası olacağını söyleyip duruyor. Bu şekerimi yükseltir mi, bebeğime zararı olur mu?</t>
         </is>
       </c>
@@ -1336,6 +1448,11 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
+          <t>Hamileliğimde gebelik şekeri çıkmıştı. Doğum yapalı 40 gün oldu, bebeğimin mevlidi var ve büyüklerim süt yapsın diye sürekli lohusa şerbeti içmemi söylüyor. Şekerim düzelmiş midir, bu şerbeti içsem bana zararı olur mu?</t>
+        </is>
+      </c>
+      <c r="F27" s="39" t="inlineStr">
+        <is>
           <t>Doğum yapalı 40 gün oldu, bebeğimin mevlidi var ve büyüklerim süt yapsın diye sürekli lohusa şerbeti içmemi söylüyor. Şekerim düzelmiş midir, bu şerbeti içsem bana zararı olur mu?</t>
         </is>
       </c>
@@ -1363,6 +1480,11 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
+          <t>Gebelik şekerim için insülin kullanmaya başladım. Haftaya bayram tatili için arabayla İzmir'den Adana'ya gideceğiz ve hava çok sıcak. Bu insülin kalemlerini yolda nasıl saklamam gerekiyor, bozulursa nasıl anlarım?</t>
+        </is>
+      </c>
+      <c r="F28" s="39" t="inlineStr">
+        <is>
           <t>İnsülin kullanmaya başladım. Haftaya bayram tatili için arabayla İzmir'den Adana'ya gideceğiz ve hava çok sıcak. Bu insülin kalemlerini yolda nasıl saklamam gerekiyor, bozulursa nasıl anlarım?</t>
         </is>
       </c>
@@ -1390,6 +1512,11 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Günde 7 kere şekerimi ölçmem gerekiyormuş ama eczaneye gittiğimde cihazın ve ölçüm çubuklarının çok pahalı olduğunu gördüm. Sağlık ocağındaki aile hekimine bu şeker ölçüm çubuklarını yazdırsam SGK tamamını karşılıyor mu?</t>
+        </is>
+      </c>
+      <c r="F29" s="39" t="inlineStr">
+        <is>
           <t>Günde 7 kere şekerimi ölçmem gerekiyormuş ama eczaneye gittiğimde cihazın ve ölçüm çubuklarının çok pahalı olduğunu gördüm. Sağlık ocağındaki aile hekimine bu şeker ölçüm çubuklarını yazdırsam SGK tamamını karşılıyor mu?</t>
         </is>
       </c>
@@ -1417,6 +1544,11 @@
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
+          <t>Gebelik şekerim için iki hafta önce insülin başladım, günde 7 kez parmak deliyorum, parmaklarım çok acıyor ve iz yapıyor. Sürekli glukoz takip cihazları (CGM) varmış, bana uygun mu, hangisini almalıyım? SGK karşılıyor mu yoksa cebimden mi alacağım?</t>
+        </is>
+      </c>
+      <c r="F30" s="39" t="inlineStr">
+        <is>
           <t>İki hafta önce insülin başladım, günde 7 kez parmak deliyorum, parmaklarım çok acıyor ve iz yapıyor. Sürekli glukoz takip cihazları (CGM) varmış, bana uygun mu, hangisini almalıyım? SGK karşılıyor mu yoksa cebimden mi alacağım?</t>
         </is>
       </c>
@@ -1444,6 +1576,11 @@
       </c>
       <c r="E31" s="22" t="inlineStr">
         <is>
+          <t>Gebelik şekerim var. Doktorum gün içinde hareketli olmamı, yemeklerden sonra yürüyüş yapmamı söyledi ama dışarı çıkacak vaktim yok. Akşam yemeğinden sonra sofrayı toplayıp, evi süpürmek ve bulaşıkları yıkamak yürüyüş, aktivite yerine geçer mi, kan şekerimi yeterince düşürür mü?</t>
+        </is>
+      </c>
+      <c r="F31" s="39" t="inlineStr">
+        <is>
           <t>Doktorum gün içinde hareketli olmamı, yemeklerden sonra yürüyüş yapmamı söyledi ama dışarı çıkacak vaktim yok. Akşam yemeğinden sonra sofrayı toplayıp, evi süpürmek ve bulaşıkları yıkamak yürüyüş, aktivite yerine geçer mi, kan şekerimi yeterince düşürür mü?</t>
         </is>
       </c>
@@ -1470,6 +1607,11 @@
         </is>
       </c>
       <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>Gebelik şekerim var. Canım inanılmaz derecede baklava çekiyor. 'Hamilelikte aşerilen şey yenmezse çocukta leke çıkar' diyorlar. Sadece bir porsiyon baklava yesem, tek seferlik yükselen şeker bebeğime zarar verir mi?</t>
+        </is>
+      </c>
+      <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Canım inanılmaz derecede baklava çekiyor. 'Hamilelikte aşerilen şey yenmezse çocukta leke çıkar' diyorlar. Sadece bir porsiyon baklava yesem, tek seferlik yükselen şeker bebeğime zarar verir mi?</t>
         </is>

</xml_diff>

<commit_message>
Q14'te hastanın kendi ifadesini geri getir, kılavuz yazımını düzelt ve API sorgu planını güncelle.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/GDM_Final_30_Soru_Birlesik.xlsx
+++ b/data/GDM_Final_30_Soru_Birlesik.xlsx
@@ -641,7 +641,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GDM ÇALIŞMASI - FİNAL 30 SORU HAVUZU (20 Hasta-Türevli + 10 Klavuz Vakası)</t>
+          <t>GDM ÇALIŞMASI - FİNAL 30 SORU HAVUZU (20 Hasta-Türevli + 10 Kılavuz Vakası)</t>
         </is>
       </c>
     </row>
@@ -703,6 +703,11 @@
           <t>Gebelik şekerim var, günlük beslenmemi nasıl düzenlemem gerekir? Ekmek, makarna gibi karbonhidratlar şekerimi yükseltiyor ama doymuyorum, neyle doyabilirim, hangi yiyeceklerden uzak durmalıyım?</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Değişiklik yok</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="65" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -954,6 +959,11 @@
           <t>Gebelik şekerim varken oruç tutabilir miyim, tutmam bebeğe zarar verir mi?</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Değişiklik yok</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="65" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1106,7 +1116,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Hamileliğimde gebelik şekeri çıktığı için bebeğim de şeker hastası olacak mı, çocukta kalıcı olur mu?</t>
+          <t>Hamileliğimde gebelik şekeri çıkmıştı. Ben şeker hastası olduğum için bebeğim de şeker hastası olacak mı, çocukta kalıcı olur mu?</t>
         </is>
       </c>
       <c r="F16" s="38" t="inlineStr">
@@ -1315,7 +1325,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -1347,7 +1357,7 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -1379,7 +1389,7 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
@@ -1395,6 +1405,11 @@
       <c r="E25" s="16" t="inlineStr">
         <is>
           <t>25 yaşındayım, 27 haftalık gebeyim. 25. haftada şeker yüklemesi yaptım, GDM çıktı. Şu an sadece diyetle takip oluyorum, insülin kullanmıyorum. Açlık şekerim genelde 88-92, tokluk 1. saatte 130-140 arasında. Ramazan'a 3 hafta var, oruç tutmak istiyorum. Tutmam ne kadar riskli, tutarsam neye dikkat etmem gerekir?</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Değişiklik yok</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1421,7 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
@@ -1422,6 +1437,11 @@
       <c r="E26" s="16" t="inlineStr">
         <is>
           <t>34 yaşındayım, 28 haftalık gebeyim. GDM tanısı aldım, günde iki kez insülin kullanıyorum (sabah ve akşam yemek öncesi). Ramazan başlıyor, oruç tutmak istiyorum. İnsülin kullanırken oruç tutmak mümkün mü, insülin dozlarımı nasıl ayarlamam gerekir, hangi durumlarda orucumu bozmalıyım?</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Değişiklik yok</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1453,7 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
@@ -1465,7 +1485,7 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
@@ -1497,7 +1517,7 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C29" s="20" t="inlineStr">
@@ -1529,7 +1549,7 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C30" s="20" t="inlineStr">
@@ -1561,7 +1581,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C31" s="22" t="inlineStr">
@@ -1593,7 +1613,7 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>Klavuz vakası</t>
+          <t>Kılavuz vakası</t>
         </is>
       </c>
       <c r="C32" s="22" t="inlineStr">
@@ -1648,6 +1668,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1661,7 +1682,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>KLAVUZ VAKA</t>
+          <t>KILAVUZ VAKA</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1860,7 +1881,7 @@
       </c>
       <c r="C4" s="36" t="inlineStr">
         <is>
-          <t>20 hasta-türevli + 10 klavuz vakası</t>
+          <t>20 hasta-türevli + 10 kılavuz vakası</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1898,7 @@
       </c>
       <c r="C5" s="36" t="inlineStr">
         <is>
-          <t>GPT (OpenAI), Claude (Anthropic), Gemini (Google), Türkçe yerli model</t>
+          <t>GPT (OpenAI), Claude (Anthropic), Gemini (Google), Trendyol-LLM-8B-T1</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1966,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Hastanın direkt sorusu simüle edilecek</t>
+          <t>Hastanın direkt sorusu simüle edilecek. Bağlam cümlesi soru metnine dahildir, ayrı bir talimat değildir.</t>
         </is>
       </c>
     </row>

</xml_diff>